<commit_message>
Fix genotype mislabeling: 14 mice corrected from HET to WT
The pipeline metadata files incorrectly labeled all pups of HET mothers
as HET. A HET x WT cross produces ~50% HET and ~50% WT offspring.
Cross-referencing with the external segmentation file (which contains
correct individual genotyping) revealed 14 mice (2,495 metadata rows)
that were mislabeled.

Changes:
- Fix Offspring Genotype in 6 metadata files (2023/2024)
- Add external data aggregation pipeline (extract_features.py)
- Add --external flag to train_classifier.py
- Add external data results and executive summary
- Update README with data correction note and external data docs

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/metadata/Data 2023 For Syl Segmentation_1.xlsx
+++ b/metadata/Data 2023 For Syl Segmentation_1.xlsx
@@ -33477,7 +33477,7 @@
       </c>
       <c r="E870" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F870" t="n">
@@ -33515,7 +33515,7 @@
       </c>
       <c r="E871" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F871" t="n">
@@ -33553,7 +33553,7 @@
       </c>
       <c r="E872" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F872" t="n">
@@ -33591,7 +33591,7 @@
       </c>
       <c r="E873" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F873" t="n">
@@ -33629,7 +33629,7 @@
       </c>
       <c r="E874" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F874" t="n">
@@ -33667,7 +33667,7 @@
       </c>
       <c r="E875" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F875" t="n">
@@ -33705,7 +33705,7 @@
       </c>
       <c r="E876" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F876" t="n">
@@ -33743,7 +33743,7 @@
       </c>
       <c r="E877" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F877" t="n">
@@ -33781,7 +33781,7 @@
       </c>
       <c r="E878" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F878" t="n">
@@ -33819,7 +33819,7 @@
       </c>
       <c r="E879" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F879" t="n">
@@ -33857,7 +33857,7 @@
       </c>
       <c r="E880" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F880" t="n">
@@ -33895,7 +33895,7 @@
       </c>
       <c r="E881" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F881" t="n">
@@ -33933,7 +33933,7 @@
       </c>
       <c r="E882" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F882" t="n">
@@ -33971,7 +33971,7 @@
       </c>
       <c r="E883" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F883" t="n">
@@ -34009,7 +34009,7 @@
       </c>
       <c r="E884" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F884" t="n">
@@ -34047,7 +34047,7 @@
       </c>
       <c r="E885" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F885" t="n">
@@ -34085,7 +34085,7 @@
       </c>
       <c r="E886" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F886" t="n">
@@ -34123,7 +34123,7 @@
       </c>
       <c r="E887" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F887" t="n">
@@ -34161,7 +34161,7 @@
       </c>
       <c r="E888" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F888" t="n">
@@ -34199,7 +34199,7 @@
       </c>
       <c r="E889" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F889" t="n">
@@ -34237,7 +34237,7 @@
       </c>
       <c r="E890" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F890" t="n">
@@ -34275,7 +34275,7 @@
       </c>
       <c r="E891" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F891" t="n">
@@ -34313,7 +34313,7 @@
       </c>
       <c r="E892" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F892" t="n">
@@ -34351,7 +34351,7 @@
       </c>
       <c r="E893" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F893" t="n">
@@ -34389,7 +34389,7 @@
       </c>
       <c r="E894" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F894" t="n">
@@ -34427,7 +34427,7 @@
       </c>
       <c r="E895" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F895" t="n">
@@ -34465,7 +34465,7 @@
       </c>
       <c r="E896" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F896" t="n">
@@ -34503,7 +34503,7 @@
       </c>
       <c r="E897" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F897" t="n">
@@ -34541,7 +34541,7 @@
       </c>
       <c r="E898" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F898" t="n">
@@ -34579,7 +34579,7 @@
       </c>
       <c r="E899" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F899" t="n">
@@ -34617,7 +34617,7 @@
       </c>
       <c r="E900" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F900" t="n">
@@ -34655,7 +34655,7 @@
       </c>
       <c r="E901" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F901" t="n">
@@ -34693,7 +34693,7 @@
       </c>
       <c r="E902" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F902" t="n">
@@ -34731,7 +34731,7 @@
       </c>
       <c r="E903" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F903" t="n">
@@ -34769,7 +34769,7 @@
       </c>
       <c r="E904" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F904" t="n">
@@ -34807,7 +34807,7 @@
       </c>
       <c r="E905" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F905" t="n">
@@ -34845,7 +34845,7 @@
       </c>
       <c r="E906" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F906" t="n">
@@ -34883,7 +34883,7 @@
       </c>
       <c r="E907" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F907" t="n">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="E908" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F908" t="n">
@@ -34959,7 +34959,7 @@
       </c>
       <c r="E909" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F909" t="n">
@@ -34997,7 +34997,7 @@
       </c>
       <c r="E910" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F910" t="n">
@@ -35035,7 +35035,7 @@
       </c>
       <c r="E911" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F911" t="n">
@@ -35073,7 +35073,7 @@
       </c>
       <c r="E912" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F912" t="n">
@@ -35111,7 +35111,7 @@
       </c>
       <c r="E913" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F913" t="n">
@@ -35149,7 +35149,7 @@
       </c>
       <c r="E914" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F914" t="n">
@@ -35187,7 +35187,7 @@
       </c>
       <c r="E915" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F915" t="n">
@@ -35225,7 +35225,7 @@
       </c>
       <c r="E916" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F916" t="n">
@@ -35263,7 +35263,7 @@
       </c>
       <c r="E917" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F917" t="n">
@@ -35301,7 +35301,7 @@
       </c>
       <c r="E918" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F918" t="n">
@@ -35339,7 +35339,7 @@
       </c>
       <c r="E919" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F919" t="n">
@@ -35377,7 +35377,7 @@
       </c>
       <c r="E920" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F920" t="n">
@@ -35415,7 +35415,7 @@
       </c>
       <c r="E921" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F921" t="n">
@@ -35453,7 +35453,7 @@
       </c>
       <c r="E922" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F922" t="n">
@@ -35491,7 +35491,7 @@
       </c>
       <c r="E923" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F923" t="n">
@@ -35529,7 +35529,7 @@
       </c>
       <c r="E924" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F924" t="n">
@@ -35567,7 +35567,7 @@
       </c>
       <c r="E925" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F925" t="n">
@@ -35605,7 +35605,7 @@
       </c>
       <c r="E926" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F926" t="n">
@@ -35643,7 +35643,7 @@
       </c>
       <c r="E927" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F927" t="n">
@@ -35681,7 +35681,7 @@
       </c>
       <c r="E928" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F928" t="n">
@@ -35719,7 +35719,7 @@
       </c>
       <c r="E929" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F929" t="n">
@@ -35757,7 +35757,7 @@
       </c>
       <c r="E930" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F930" t="n">
@@ -35795,7 +35795,7 @@
       </c>
       <c r="E931" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F931" t="n">
@@ -35833,7 +35833,7 @@
       </c>
       <c r="E932" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F932" t="n">
@@ -35871,7 +35871,7 @@
       </c>
       <c r="E933" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F933" t="n">
@@ -35909,7 +35909,7 @@
       </c>
       <c r="E934" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F934" t="n">
@@ -35947,7 +35947,7 @@
       </c>
       <c r="E935" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F935" t="n">
@@ -35985,7 +35985,7 @@
       </c>
       <c r="E936" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F936" t="n">
@@ -36023,7 +36023,7 @@
       </c>
       <c r="E937" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F937" t="n">
@@ -36061,7 +36061,7 @@
       </c>
       <c r="E938" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F938" t="n">
@@ -36099,7 +36099,7 @@
       </c>
       <c r="E939" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F939" t="n">
@@ -36137,7 +36137,7 @@
       </c>
       <c r="E940" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F940" t="n">
@@ -36175,7 +36175,7 @@
       </c>
       <c r="E941" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F941" t="n">
@@ -36213,7 +36213,7 @@
       </c>
       <c r="E942" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F942" t="n">
@@ -36251,7 +36251,7 @@
       </c>
       <c r="E943" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F943" t="n">
@@ -36289,7 +36289,7 @@
       </c>
       <c r="E944" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F944" t="n">
@@ -36327,7 +36327,7 @@
       </c>
       <c r="E945" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F945" t="n">
@@ -36365,7 +36365,7 @@
       </c>
       <c r="E946" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F946" t="n">
@@ -36403,7 +36403,7 @@
       </c>
       <c r="E947" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F947" t="n">
@@ -36441,7 +36441,7 @@
       </c>
       <c r="E948" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F948" t="n">
@@ -36479,7 +36479,7 @@
       </c>
       <c r="E949" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F949" t="n">
@@ -36517,7 +36517,7 @@
       </c>
       <c r="E950" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F950" t="n">
@@ -36555,7 +36555,7 @@
       </c>
       <c r="E951" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F951" t="n">
@@ -36593,7 +36593,7 @@
       </c>
       <c r="E952" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F952" t="n">
@@ -36631,7 +36631,7 @@
       </c>
       <c r="E953" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F953" t="n">
@@ -36669,7 +36669,7 @@
       </c>
       <c r="E954" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F954" t="n">
@@ -36707,7 +36707,7 @@
       </c>
       <c r="E955" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F955" t="n">
@@ -36745,7 +36745,7 @@
       </c>
       <c r="E956" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F956" t="n">
@@ -36783,7 +36783,7 @@
       </c>
       <c r="E957" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F957" t="n">
@@ -36821,7 +36821,7 @@
       </c>
       <c r="E958" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F958" t="n">
@@ -36859,7 +36859,7 @@
       </c>
       <c r="E959" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F959" t="n">
@@ -36897,7 +36897,7 @@
       </c>
       <c r="E960" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F960" t="n">
@@ -36935,7 +36935,7 @@
       </c>
       <c r="E961" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F961" t="n">
@@ -36973,7 +36973,7 @@
       </c>
       <c r="E962" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F962" t="n">
@@ -37011,7 +37011,7 @@
       </c>
       <c r="E963" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F963" t="n">
@@ -37049,7 +37049,7 @@
       </c>
       <c r="E964" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F964" t="n">
@@ -37087,7 +37087,7 @@
       </c>
       <c r="E965" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F965" t="n">
@@ -37125,7 +37125,7 @@
       </c>
       <c r="E966" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F966" t="n">
@@ -37163,7 +37163,7 @@
       </c>
       <c r="E967" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F967" t="n">
@@ -37201,7 +37201,7 @@
       </c>
       <c r="E968" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F968" t="n">
@@ -37239,7 +37239,7 @@
       </c>
       <c r="E969" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F969" t="n">
@@ -37277,7 +37277,7 @@
       </c>
       <c r="E970" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F970" t="n">
@@ -37315,7 +37315,7 @@
       </c>
       <c r="E971" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F971" t="n">
@@ -37353,7 +37353,7 @@
       </c>
       <c r="E972" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F972" t="n">
@@ -37391,7 +37391,7 @@
       </c>
       <c r="E973" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F973" t="n">
@@ -37429,7 +37429,7 @@
       </c>
       <c r="E974" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F974" t="n">
@@ -37467,7 +37467,7 @@
       </c>
       <c r="E975" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F975" t="n">
@@ -37505,7 +37505,7 @@
       </c>
       <c r="E976" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F976" t="n">
@@ -37543,7 +37543,7 @@
       </c>
       <c r="E977" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F977" t="n">
@@ -37581,7 +37581,7 @@
       </c>
       <c r="E978" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F978" t="n">
@@ -37619,7 +37619,7 @@
       </c>
       <c r="E979" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F979" t="n">
@@ -37657,7 +37657,7 @@
       </c>
       <c r="E980" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F980" t="n">
@@ -37695,7 +37695,7 @@
       </c>
       <c r="E981" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F981" t="n">
@@ -37733,7 +37733,7 @@
       </c>
       <c r="E982" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F982" t="n">
@@ -37771,7 +37771,7 @@
       </c>
       <c r="E983" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F983" t="n">
@@ -37809,7 +37809,7 @@
       </c>
       <c r="E984" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F984" t="n">
@@ -37847,7 +37847,7 @@
       </c>
       <c r="E985" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F985" t="n">
@@ -37885,7 +37885,7 @@
       </c>
       <c r="E986" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F986" t="n">
@@ -37923,7 +37923,7 @@
       </c>
       <c r="E987" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F987" t="n">
@@ -37961,7 +37961,7 @@
       </c>
       <c r="E988" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F988" t="n">
@@ -37999,7 +37999,7 @@
       </c>
       <c r="E989" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F989" t="n">
@@ -38037,7 +38037,7 @@
       </c>
       <c r="E990" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F990" t="n">
@@ -38075,7 +38075,7 @@
       </c>
       <c r="E991" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F991" t="n">
@@ -38113,7 +38113,7 @@
       </c>
       <c r="E992" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F992" t="n">
@@ -38151,7 +38151,7 @@
       </c>
       <c r="E993" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F993" t="n">
@@ -38189,7 +38189,7 @@
       </c>
       <c r="E994" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F994" t="n">
@@ -38227,7 +38227,7 @@
       </c>
       <c r="E995" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F995" t="n">
@@ -38265,7 +38265,7 @@
       </c>
       <c r="E996" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F996" t="n">
@@ -38303,7 +38303,7 @@
       </c>
       <c r="E997" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F997" t="n">
@@ -38341,7 +38341,7 @@
       </c>
       <c r="E998" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F998" t="n">
@@ -38379,7 +38379,7 @@
       </c>
       <c r="E999" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F999" t="n">
@@ -38417,7 +38417,7 @@
       </c>
       <c r="E1000" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1000" t="n">
@@ -38455,7 +38455,7 @@
       </c>
       <c r="E1001" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1001" t="n">
@@ -38493,7 +38493,7 @@
       </c>
       <c r="E1002" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1002" t="n">
@@ -38531,7 +38531,7 @@
       </c>
       <c r="E1003" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1003" t="n">
@@ -38569,7 +38569,7 @@
       </c>
       <c r="E1004" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1004" t="n">
@@ -38607,7 +38607,7 @@
       </c>
       <c r="E1005" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1005" t="n">
@@ -38645,7 +38645,7 @@
       </c>
       <c r="E1006" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1006" t="n">
@@ -38683,7 +38683,7 @@
       </c>
       <c r="E1007" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1007" t="n">
@@ -38721,7 +38721,7 @@
       </c>
       <c r="E1008" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1008" t="n">
@@ -38759,7 +38759,7 @@
       </c>
       <c r="E1009" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1009" t="n">
@@ -38797,7 +38797,7 @@
       </c>
       <c r="E1010" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1010" t="n">
@@ -38835,7 +38835,7 @@
       </c>
       <c r="E1011" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1011" t="n">
@@ -38873,7 +38873,7 @@
       </c>
       <c r="E1012" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1012" t="n">
@@ -38911,7 +38911,7 @@
       </c>
       <c r="E1013" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1013" t="n">
@@ -38949,7 +38949,7 @@
       </c>
       <c r="E1014" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1014" t="n">
@@ -38987,7 +38987,7 @@
       </c>
       <c r="E1015" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1015" t="n">
@@ -39025,7 +39025,7 @@
       </c>
       <c r="E1016" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1016" t="n">
@@ -39063,7 +39063,7 @@
       </c>
       <c r="E1017" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1017" t="n">
@@ -39101,7 +39101,7 @@
       </c>
       <c r="E1018" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1018" t="n">
@@ -39139,7 +39139,7 @@
       </c>
       <c r="E1019" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1019" t="n">
@@ -39177,7 +39177,7 @@
       </c>
       <c r="E1020" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1020" t="n">
@@ -39215,7 +39215,7 @@
       </c>
       <c r="E1021" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1021" t="n">
@@ -39253,7 +39253,7 @@
       </c>
       <c r="E1022" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1022" t="n">
@@ -39291,7 +39291,7 @@
       </c>
       <c r="E1023" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1023" t="n">
@@ -39329,7 +39329,7 @@
       </c>
       <c r="E1024" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1024" t="n">
@@ -39367,7 +39367,7 @@
       </c>
       <c r="E1025" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1025" t="n">
@@ -39405,7 +39405,7 @@
       </c>
       <c r="E1026" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1026" t="n">
@@ -39443,7 +39443,7 @@
       </c>
       <c r="E1027" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1027" t="n">
@@ -39481,7 +39481,7 @@
       </c>
       <c r="E1028" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1028" t="n">
@@ -39519,7 +39519,7 @@
       </c>
       <c r="E1029" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1029" t="n">
@@ -39557,7 +39557,7 @@
       </c>
       <c r="E1030" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1030" t="n">
@@ -39595,7 +39595,7 @@
       </c>
       <c r="E1031" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1031" t="n">
@@ -39633,7 +39633,7 @@
       </c>
       <c r="E1032" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1032" t="n">
@@ -39671,7 +39671,7 @@
       </c>
       <c r="E1033" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1033" t="n">
@@ -39709,7 +39709,7 @@
       </c>
       <c r="E1034" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1034" t="n">
@@ -39747,7 +39747,7 @@
       </c>
       <c r="E1035" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1035" t="n">
@@ -39785,7 +39785,7 @@
       </c>
       <c r="E1036" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1036" t="n">
@@ -39823,7 +39823,7 @@
       </c>
       <c r="E1037" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1037" t="n">
@@ -39861,7 +39861,7 @@
       </c>
       <c r="E1038" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1038" t="n">
@@ -39899,7 +39899,7 @@
       </c>
       <c r="E1039" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1039" t="n">
@@ -39937,7 +39937,7 @@
       </c>
       <c r="E1040" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1040" t="n">
@@ -39975,7 +39975,7 @@
       </c>
       <c r="E1041" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1041" t="n">
@@ -40013,7 +40013,7 @@
       </c>
       <c r="E1042" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1042" t="n">
@@ -40051,7 +40051,7 @@
       </c>
       <c r="E1043" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1043" t="n">
@@ -40089,7 +40089,7 @@
       </c>
       <c r="E1044" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1044" t="n">
@@ -40127,7 +40127,7 @@
       </c>
       <c r="E1045" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1045" t="n">
@@ -40165,7 +40165,7 @@
       </c>
       <c r="E1046" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1046" t="n">
@@ -40203,7 +40203,7 @@
       </c>
       <c r="E1047" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1047" t="n">
@@ -40241,7 +40241,7 @@
       </c>
       <c r="E1048" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1048" t="n">
@@ -40279,7 +40279,7 @@
       </c>
       <c r="E1049" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1049" t="n">
@@ -40317,7 +40317,7 @@
       </c>
       <c r="E1050" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1050" t="n">
@@ -40355,7 +40355,7 @@
       </c>
       <c r="E1051" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1051" t="n">
@@ -40393,7 +40393,7 @@
       </c>
       <c r="E1052" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1052" t="n">
@@ -40431,7 +40431,7 @@
       </c>
       <c r="E1053" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1053" t="n">
@@ -40469,7 +40469,7 @@
       </c>
       <c r="E1054" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1054" t="n">
@@ -40507,7 +40507,7 @@
       </c>
       <c r="E1055" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1055" t="n">
@@ -40545,7 +40545,7 @@
       </c>
       <c r="E1056" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1056" t="n">
@@ -40583,7 +40583,7 @@
       </c>
       <c r="E1057" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1057" t="n">
@@ -40621,7 +40621,7 @@
       </c>
       <c r="E1058" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1058" t="n">
@@ -40659,7 +40659,7 @@
       </c>
       <c r="E1059" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1059" t="n">
@@ -40697,7 +40697,7 @@
       </c>
       <c r="E1060" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1060" t="n">
@@ -40735,7 +40735,7 @@
       </c>
       <c r="E1061" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1061" t="n">
@@ -40773,7 +40773,7 @@
       </c>
       <c r="E1062" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1062" t="n">
@@ -40811,7 +40811,7 @@
       </c>
       <c r="E1063" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1063" t="n">
@@ -40849,7 +40849,7 @@
       </c>
       <c r="E1064" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1064" t="n">
@@ -40887,7 +40887,7 @@
       </c>
       <c r="E1065" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1065" t="n">
@@ -40925,7 +40925,7 @@
       </c>
       <c r="E1066" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1066" t="n">
@@ -40963,7 +40963,7 @@
       </c>
       <c r="E1067" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1067" t="n">
@@ -41001,7 +41001,7 @@
       </c>
       <c r="E1068" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1068" t="n">
@@ -41039,7 +41039,7 @@
       </c>
       <c r="E1069" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1069" t="n">
@@ -41077,7 +41077,7 @@
       </c>
       <c r="E1070" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1070" t="n">
@@ -41115,7 +41115,7 @@
       </c>
       <c r="E1071" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1071" t="n">
@@ -41153,7 +41153,7 @@
       </c>
       <c r="E1072" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1072" t="n">
@@ -41191,7 +41191,7 @@
       </c>
       <c r="E1073" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1073" t="n">
@@ -41229,7 +41229,7 @@
       </c>
       <c r="E1074" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1074" t="n">
@@ -41267,7 +41267,7 @@
       </c>
       <c r="E1075" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1075" t="n">
@@ -41305,7 +41305,7 @@
       </c>
       <c r="E1076" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1076" t="n">
@@ -41343,7 +41343,7 @@
       </c>
       <c r="E1077" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1077" t="n">
@@ -41381,7 +41381,7 @@
       </c>
       <c r="E1078" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1078" t="n">
@@ -41419,7 +41419,7 @@
       </c>
       <c r="E1079" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1079" t="n">
@@ -41457,7 +41457,7 @@
       </c>
       <c r="E1080" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1080" t="n">
@@ -41495,7 +41495,7 @@
       </c>
       <c r="E1081" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1081" t="n">
@@ -41533,7 +41533,7 @@
       </c>
       <c r="E1082" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1082" t="n">
@@ -41571,7 +41571,7 @@
       </c>
       <c r="E1083" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1083" t="n">
@@ -41609,7 +41609,7 @@
       </c>
       <c r="E1084" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1084" t="n">
@@ -41647,7 +41647,7 @@
       </c>
       <c r="E1085" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1085" t="n">
@@ -41685,7 +41685,7 @@
       </c>
       <c r="E1086" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1086" t="n">
@@ -41723,7 +41723,7 @@
       </c>
       <c r="E1087" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1087" t="n">
@@ -41761,7 +41761,7 @@
       </c>
       <c r="E1088" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1088" t="n">
@@ -41799,7 +41799,7 @@
       </c>
       <c r="E1089" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1089" t="n">
@@ -41837,7 +41837,7 @@
       </c>
       <c r="E1090" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1090" t="n">
@@ -41875,7 +41875,7 @@
       </c>
       <c r="E1091" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1091" t="n">
@@ -41913,7 +41913,7 @@
       </c>
       <c r="E1092" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1092" t="n">
@@ -41951,7 +41951,7 @@
       </c>
       <c r="E1093" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1093" t="n">
@@ -41989,7 +41989,7 @@
       </c>
       <c r="E1094" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1094" t="n">
@@ -42027,7 +42027,7 @@
       </c>
       <c r="E1095" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1095" t="n">
@@ -42065,7 +42065,7 @@
       </c>
       <c r="E1096" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1096" t="n">
@@ -42103,7 +42103,7 @@
       </c>
       <c r="E1097" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1097" t="n">
@@ -42141,7 +42141,7 @@
       </c>
       <c r="E1098" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1098" t="n">
@@ -42179,7 +42179,7 @@
       </c>
       <c r="E1099" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1099" t="n">
@@ -42217,7 +42217,7 @@
       </c>
       <c r="E1100" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1100" t="n">
@@ -42255,7 +42255,7 @@
       </c>
       <c r="E1101" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1101" t="n">
@@ -42293,7 +42293,7 @@
       </c>
       <c r="E1102" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1102" t="n">
@@ -42331,7 +42331,7 @@
       </c>
       <c r="E1103" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1103" t="n">
@@ -42369,7 +42369,7 @@
       </c>
       <c r="E1104" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1104" t="n">
@@ -42407,7 +42407,7 @@
       </c>
       <c r="E1105" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1105" t="n">
@@ -42445,7 +42445,7 @@
       </c>
       <c r="E1106" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1106" t="n">
@@ -42483,7 +42483,7 @@
       </c>
       <c r="E1107" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1107" t="n">
@@ -42521,7 +42521,7 @@
       </c>
       <c r="E1108" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1108" t="n">
@@ -42559,7 +42559,7 @@
       </c>
       <c r="E1109" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1109" t="n">
@@ -42597,7 +42597,7 @@
       </c>
       <c r="E1110" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1110" t="n">
@@ -42635,7 +42635,7 @@
       </c>
       <c r="E1111" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1111" t="n">
@@ -42673,7 +42673,7 @@
       </c>
       <c r="E1112" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1112" t="n">
@@ -42711,7 +42711,7 @@
       </c>
       <c r="E1113" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1113" t="n">
@@ -42749,7 +42749,7 @@
       </c>
       <c r="E1114" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1114" t="n">
@@ -42787,7 +42787,7 @@
       </c>
       <c r="E1115" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1115" t="n">
@@ -42825,7 +42825,7 @@
       </c>
       <c r="E1116" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1116" t="n">
@@ -42863,7 +42863,7 @@
       </c>
       <c r="E1117" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1117" t="n">
@@ -42901,7 +42901,7 @@
       </c>
       <c r="E1118" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1118" t="n">
@@ -42939,7 +42939,7 @@
       </c>
       <c r="E1119" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1119" t="n">
@@ -42977,7 +42977,7 @@
       </c>
       <c r="E1120" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1120" t="n">
@@ -43015,7 +43015,7 @@
       </c>
       <c r="E1121" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1121" t="n">
@@ -43053,7 +43053,7 @@
       </c>
       <c r="E1122" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1122" t="n">
@@ -43091,7 +43091,7 @@
       </c>
       <c r="E1123" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1123" t="n">
@@ -43129,7 +43129,7 @@
       </c>
       <c r="E1124" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1124" t="n">
@@ -43167,7 +43167,7 @@
       </c>
       <c r="E1125" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1125" t="n">
@@ -43205,7 +43205,7 @@
       </c>
       <c r="E1126" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1126" t="n">
@@ -43243,7 +43243,7 @@
       </c>
       <c r="E1127" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1127" t="n">
@@ -43281,7 +43281,7 @@
       </c>
       <c r="E1128" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1128" t="n">
@@ -43319,7 +43319,7 @@
       </c>
       <c r="E1129" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1129" t="n">
@@ -43357,7 +43357,7 @@
       </c>
       <c r="E1130" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1130" t="n">
@@ -43395,7 +43395,7 @@
       </c>
       <c r="E1131" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1131" t="n">
@@ -43433,7 +43433,7 @@
       </c>
       <c r="E1132" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1132" t="n">
@@ -43471,7 +43471,7 @@
       </c>
       <c r="E1133" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1133" t="n">
@@ -43509,7 +43509,7 @@
       </c>
       <c r="E1134" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1134" t="n">
@@ -43547,7 +43547,7 @@
       </c>
       <c r="E1135" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1135" t="n">
@@ -43585,7 +43585,7 @@
       </c>
       <c r="E1136" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1136" t="n">
@@ -43623,7 +43623,7 @@
       </c>
       <c r="E1137" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1137" t="n">
@@ -43661,7 +43661,7 @@
       </c>
       <c r="E1138" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1138" t="n">
@@ -43699,7 +43699,7 @@
       </c>
       <c r="E1139" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1139" t="n">
@@ -43737,7 +43737,7 @@
       </c>
       <c r="E1140" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1140" t="n">
@@ -43775,7 +43775,7 @@
       </c>
       <c r="E1141" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1141" t="n">
@@ -43813,7 +43813,7 @@
       </c>
       <c r="E1142" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1142" t="n">
@@ -43851,7 +43851,7 @@
       </c>
       <c r="E1143" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1143" t="n">
@@ -43889,7 +43889,7 @@
       </c>
       <c r="E1144" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1144" t="n">
@@ -43927,7 +43927,7 @@
       </c>
       <c r="E1145" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1145" t="n">
@@ -43965,7 +43965,7 @@
       </c>
       <c r="E1146" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1146" t="n">
@@ -44003,7 +44003,7 @@
       </c>
       <c r="E1147" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1147" t="n">
@@ -44041,7 +44041,7 @@
       </c>
       <c r="E1148" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1148" t="n">
@@ -44079,7 +44079,7 @@
       </c>
       <c r="E1149" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1149" t="n">
@@ -44117,7 +44117,7 @@
       </c>
       <c r="E1150" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1150" t="n">
@@ -44155,7 +44155,7 @@
       </c>
       <c r="E1151" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1151" t="n">
@@ -44193,7 +44193,7 @@
       </c>
       <c r="E1152" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1152" t="n">
@@ -44231,7 +44231,7 @@
       </c>
       <c r="E1153" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1153" t="n">
@@ -44269,7 +44269,7 @@
       </c>
       <c r="E1154" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1154" t="n">
@@ -44307,7 +44307,7 @@
       </c>
       <c r="E1155" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1155" t="n">
@@ -44345,7 +44345,7 @@
       </c>
       <c r="E1156" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1156" t="n">
@@ -44383,7 +44383,7 @@
       </c>
       <c r="E1157" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1157" t="n">
@@ -44421,7 +44421,7 @@
       </c>
       <c r="E1158" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1158" t="n">
@@ -44459,7 +44459,7 @@
       </c>
       <c r="E1159" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1159" t="n">
@@ -44497,7 +44497,7 @@
       </c>
       <c r="E1160" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1160" t="n">
@@ -44535,7 +44535,7 @@
       </c>
       <c r="E1161" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1161" t="n">
@@ -44573,7 +44573,7 @@
       </c>
       <c r="E1162" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1162" t="n">
@@ -44611,7 +44611,7 @@
       </c>
       <c r="E1163" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1163" t="n">
@@ -44649,7 +44649,7 @@
       </c>
       <c r="E1164" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1164" t="n">
@@ -44687,7 +44687,7 @@
       </c>
       <c r="E1165" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1165" t="n">
@@ -44725,7 +44725,7 @@
       </c>
       <c r="E1166" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1166" t="n">
@@ -44763,7 +44763,7 @@
       </c>
       <c r="E1167" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1167" t="n">
@@ -44801,7 +44801,7 @@
       </c>
       <c r="E1168" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1168" t="n">
@@ -44839,7 +44839,7 @@
       </c>
       <c r="E1169" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1169" t="n">
@@ -44877,7 +44877,7 @@
       </c>
       <c r="E1170" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1170" t="n">
@@ -44915,7 +44915,7 @@
       </c>
       <c r="E1171" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1171" t="n">
@@ -44953,7 +44953,7 @@
       </c>
       <c r="E1172" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1172" t="n">
@@ -44991,7 +44991,7 @@
       </c>
       <c r="E1173" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1173" t="n">
@@ -45029,7 +45029,7 @@
       </c>
       <c r="E1174" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1174" t="n">
@@ -45067,7 +45067,7 @@
       </c>
       <c r="E1175" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1175" t="n">
@@ -45105,7 +45105,7 @@
       </c>
       <c r="E1176" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1176" t="n">
@@ -45143,7 +45143,7 @@
       </c>
       <c r="E1177" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1177" t="n">
@@ -45181,7 +45181,7 @@
       </c>
       <c r="E1178" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1178" t="n">
@@ -45219,7 +45219,7 @@
       </c>
       <c r="E1179" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1179" t="n">
@@ -45257,7 +45257,7 @@
       </c>
       <c r="E1180" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1180" t="n">
@@ -45295,7 +45295,7 @@
       </c>
       <c r="E1181" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1181" t="n">
@@ -45333,7 +45333,7 @@
       </c>
       <c r="E1182" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1182" t="n">
@@ -45371,7 +45371,7 @@
       </c>
       <c r="E1183" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1183" t="n">
@@ -45409,7 +45409,7 @@
       </c>
       <c r="E1184" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1184" t="n">
@@ -45447,7 +45447,7 @@
       </c>
       <c r="E1185" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1185" t="n">
@@ -45485,7 +45485,7 @@
       </c>
       <c r="E1186" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1186" t="n">
@@ -45523,7 +45523,7 @@
       </c>
       <c r="E1187" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1187" t="n">
@@ -45561,7 +45561,7 @@
       </c>
       <c r="E1188" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1188" t="n">
@@ -45599,7 +45599,7 @@
       </c>
       <c r="E1189" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1189" t="n">
@@ -45637,7 +45637,7 @@
       </c>
       <c r="E1190" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1190" t="n">
@@ -45675,7 +45675,7 @@
       </c>
       <c r="E1191" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1191" t="n">
@@ -45713,7 +45713,7 @@
       </c>
       <c r="E1192" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1192" t="n">
@@ -45751,7 +45751,7 @@
       </c>
       <c r="E1193" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1193" t="n">
@@ -45789,7 +45789,7 @@
       </c>
       <c r="E1194" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1194" t="n">
@@ -45827,7 +45827,7 @@
       </c>
       <c r="E1195" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1195" t="n">
@@ -45865,7 +45865,7 @@
       </c>
       <c r="E1196" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1196" t="n">
@@ -45903,7 +45903,7 @@
       </c>
       <c r="E1197" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1197" t="n">
@@ -45941,7 +45941,7 @@
       </c>
       <c r="E1198" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1198" t="n">
@@ -45979,7 +45979,7 @@
       </c>
       <c r="E1199" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1199" t="n">
@@ -46017,7 +46017,7 @@
       </c>
       <c r="E1200" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1200" t="n">
@@ -46055,7 +46055,7 @@
       </c>
       <c r="E1201" t="inlineStr">
         <is>
-          <t>HET</t>
+          <t>WT</t>
         </is>
       </c>
       <c r="F1201" t="n">

</xml_diff>